<commit_message>
Fixed rotation in data generatioin
</commit_message>
<xml_diff>
--- a/Program's/Data_generation_settings.xlsx
+++ b/Program's/Data_generation_settings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hogeschoolutrecht.sharepoint.com/sites/int_Onderwijs_mnleprojectimagine/Gedeelde documenten/DataProgram/Program's/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="149" documentId="8_{EBE526E8-301D-439D-BBD0-DDC04C017095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9E73108-52D2-47DF-A69B-9CF53A07C891}"/>
+  <xr:revisionPtr revIDLastSave="208" documentId="8_{EBE526E8-301D-439D-BBD0-DDC04C017095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E9CB2BD-CEEF-4720-8B7D-F76F219DE81F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{40F60AC9-7D5C-4796-9560-5C6031084052}"/>
+    <workbookView xWindow="7665" yWindow="4560" windowWidth="28800" windowHeight="15345" activeTab="3" xr2:uid="{40F60AC9-7D5C-4796-9560-5C6031084052}"/>
   </bookViews>
   <sheets>
     <sheet name="Sensors" sheetId="1" r:id="rId1"/>
@@ -2021,10 +2021,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C690120A-A78E-48C8-BF8E-8A7A03B41FAF}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="1" max="1" width="38.140625" customWidth="1"/>
     <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -2070,7 +2070,7 @@
         <v>1.5</v>
       </c>
       <c r="E2" s="1">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F2" s="1">
         <v>0</v>
@@ -2102,7 +2102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>34</v>
       </c>
@@ -2124,6 +2124,15 @@
       <c r="G4" s="9">
         <v>45</v>
       </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="6"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2191,16 +2200,16 @@
         <v>42</v>
       </c>
       <c r="B3" s="1">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="C3" s="1">
         <v>0.2</v>
       </c>
       <c r="D3" s="1">
-        <v>1.0000000000000001E-5</v>
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="E3" s="1">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F3" s="1">
         <v>1E-3</v>
@@ -2220,7 +2229,7 @@
         <v>9.9999999999999995E-7</v>
       </c>
       <c r="E4" s="1">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="F4" s="1">
         <v>1E-3</v>
@@ -2231,7 +2240,7 @@
         <v>43</v>
       </c>
       <c r="B5" s="7">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C5" s="7">
         <v>0.01</v>
@@ -2267,9 +2276,11 @@
     <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -2321,10 +2332,7 @@
       <c r="C2" t="s">
         <v>43</v>
       </c>
-      <c r="H2" t="s">
-        <v>48</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="D2" t="s">
         <v>48</v>
       </c>
       <c r="J2" t="s">
@@ -2342,7 +2350,7 @@
         <v>58</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -2350,10 +2358,13 @@
       <c r="D3" t="s">
         <v>48</v>
       </c>
-      <c r="I3" t="s">
-        <v>48</v>
-      </c>
-      <c r="L3" t="s">
+      <c r="G3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J3" t="s">
+        <v>48</v>
+      </c>
+      <c r="K3" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2400,7 +2411,7 @@
         <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C5" t="s">
         <v>42</v>
@@ -2438,7 +2449,7 @@
         <v>54</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C6" t="s">
         <v>52</v>
@@ -2495,6 +2506,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="1fc8c048-acb1-4bfa-b76d-dd24d91bfa45" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6864db5e-2ba5-43d3-9971-5f9c69543783">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003423A5F209A89D4CB19EEA099B551A17" ma:contentTypeVersion="11" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="7890ff3c720bac6bb85ddf3222d137c1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6864db5e-2ba5-43d3-9971-5f9c69543783" xmlns:ns3="1fc8c048-acb1-4bfa-b76d-dd24d91bfa45" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb943a136b0a67757f8c603298115e36" ns2:_="" ns3:_="">
     <xsd:import namespace="6864db5e-2ba5-43d3-9971-5f9c69543783"/>
@@ -2689,27 +2720,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B17E3705-3D87-4528-A7DE-60BD1D086448}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="1fc8c048-acb1-4bfa-b76d-dd24d91bfa45" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6864db5e-2ba5-43d3-9971-5f9c69543783">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{852BFB73-ED99-461A-AA7A-A090EF1DA3A2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="1fc8c048-acb1-4bfa-b76d-dd24d91bfa45"/>
+    <ds:schemaRef ds:uri="6864db5e-2ba5-43d3-9971-5f9c69543783"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7C7159D-9BEA-4379-830F-4F3D0CA1B308}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2726,23 +2756,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B17E3705-3D87-4528-A7DE-60BD1D086448}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{852BFB73-ED99-461A-AA7A-A090EF1DA3A2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="1fc8c048-acb1-4bfa-b76d-dd24d91bfa45"/>
-    <ds:schemaRef ds:uri="6864db5e-2ba5-43d3-9971-5f9c69543783"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Clouds for noice test and explinatioins in analyser
</commit_message>
<xml_diff>
--- a/Program's/Data_generation_settings.xlsx
+++ b/Program's/Data_generation_settings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hogeschoolutrecht.sharepoint.com/sites/int_Onderwijs_mnleprojectimagine/Gedeelde documenten/DataProgram/Program's/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="8_{EBE526E8-301D-439D-BBD0-DDC04C017095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E9CB2BD-CEEF-4720-8B7D-F76F219DE81F}"/>
+  <xr:revisionPtr revIDLastSave="244" documentId="8_{EBE526E8-301D-439D-BBD0-DDC04C017095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C20AD30C-A320-4DCB-B19F-2B94E8B0D285}"/>
   <bookViews>
-    <workbookView xWindow="7665" yWindow="4560" windowWidth="28800" windowHeight="15345" activeTab="3" xr2:uid="{40F60AC9-7D5C-4796-9560-5C6031084052}"/>
+    <workbookView xWindow="8355" yWindow="5250" windowWidth="28800" windowHeight="15345" activeTab="2" xr2:uid="{40F60AC9-7D5C-4796-9560-5C6031084052}"/>
   </bookViews>
   <sheets>
     <sheet name="Sensors" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="59">
   <si>
     <t>sensor_id</t>
   </si>
@@ -109,18 +109,12 @@
     <t>100.0</t>
   </si>
   <si>
-    <t>0.02</t>
-  </si>
-  <si>
     <t>lidar_os1</t>
   </si>
   <si>
     <t>120.0</t>
   </si>
   <si>
-    <t>0.01</t>
-  </si>
-  <si>
     <t>low_res_test</t>
   </si>
   <si>
@@ -130,18 +124,12 @@
     <t>5.0</t>
   </si>
   <si>
-    <t>0.05</t>
-  </si>
-  <si>
     <t>high_prec</t>
   </si>
   <si>
     <t>50.0</t>
   </si>
   <si>
-    <t>0.000</t>
-  </si>
-  <si>
     <t>config_id</t>
   </si>
   <si>
@@ -242,6 +230,18 @@
   </si>
   <si>
     <t>Test_fast</t>
+  </si>
+  <si>
+    <t>Basler_ace_2_0,0001_noice</t>
+  </si>
+  <si>
+    <t>Basler_ace_2_0,00005_noice</t>
+  </si>
+  <si>
+    <t>Basler_ace_2_0,0005_noice</t>
+  </si>
+  <si>
+    <t>Test_basler_noice</t>
   </si>
 </sst>
 </file>
@@ -1452,8 +1452,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1FB33333-3360-4578-86D6-9896CBB35280}" name="sensors" displayName="sensors" ref="A1:H7" totalsRowShown="0" headerRowDxfId="37" dataDxfId="35" headerRowBorderDxfId="36" tableBorderDxfId="34" totalsRowBorderDxfId="33">
-  <autoFilter ref="A1:H7" xr:uid="{1FB33333-3360-4578-86D6-9896CBB35280}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1FB33333-3360-4578-86D6-9896CBB35280}" name="sensors" displayName="sensors" ref="A1:H10" totalsRowShown="0" headerRowDxfId="37" dataDxfId="35" headerRowBorderDxfId="36" tableBorderDxfId="34" totalsRowBorderDxfId="33">
+  <autoFilter ref="A1:H10" xr:uid="{1FB33333-3360-4578-86D6-9896CBB35280}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{72190787-3DD2-4A96-97E4-9D7020BA3D7F}" name="sensor_id" dataDxfId="32"/>
     <tableColumn id="2" xr3:uid="{DF6A5913-E7E9-49FE-A4B6-AAA8FC11EDFE}" name="type" dataDxfId="31"/>
@@ -1816,7 +1816,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{059D14D0-AE04-4573-838F-73D4AC3A9BF2}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.42578125" customWidth="1"/>
@@ -1903,13 +1903,13 @@
       <c r="G3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>14</v>
+      <c r="H3" s="1">
+        <v>2E-3</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>12</v>
@@ -1927,18 +1927,18 @@
         <v>45</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
+      </c>
+      <c r="H4" s="1">
+        <v>1E-3</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C5" s="1">
         <v>64</v>
@@ -1953,18 +1953,18 @@
         <v>60</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
+      </c>
+      <c r="H5" s="1">
+        <v>5.0000000000000001E-4</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C6" s="7">
         <v>1024</v>
@@ -1979,21 +1979,21 @@
         <v>90</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>24</v>
+        <v>20</v>
+      </c>
+      <c r="H6" s="7">
+        <v>1.0000000000000001E-5</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D7" s="11">
         <v>1944</v>
@@ -2009,6 +2009,84 @@
       </c>
       <c r="H7" s="7">
         <v>1E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="7">
+        <v>1944</v>
+      </c>
+      <c r="E8" s="7">
+        <v>70</v>
+      </c>
+      <c r="F8" s="7">
+        <v>60</v>
+      </c>
+      <c r="G8" s="7">
+        <v>10</v>
+      </c>
+      <c r="H8" s="7">
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="7">
+        <v>1944</v>
+      </c>
+      <c r="E9" s="7">
+        <v>70</v>
+      </c>
+      <c r="F9" s="7">
+        <v>60</v>
+      </c>
+      <c r="G9" s="7">
+        <v>10</v>
+      </c>
+      <c r="H9" s="7">
+        <v>5.0000000000000001E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="7">
+        <v>1944</v>
+      </c>
+      <c r="E10" s="7">
+        <v>70</v>
+      </c>
+      <c r="F10" s="7">
+        <v>60</v>
+      </c>
+      <c r="G10" s="7">
+        <v>10</v>
+      </c>
+      <c r="H10" s="7">
+        <v>5.0000000000000002E-5</v>
       </c>
     </row>
   </sheetData>
@@ -2035,30 +2113,30 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B2" s="1">
         <v>0</v>
@@ -2081,7 +2159,7 @@
     </row>
     <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B3" s="1">
         <v>0</v>
@@ -2104,7 +2182,7 @@
     </row>
     <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B4" s="7">
         <v>2</v>
@@ -2157,27 +2235,27 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B2" s="1">
         <v>100</v>
@@ -2197,10 +2275,10 @@
     </row>
     <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B3" s="1">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="C3" s="1">
         <v>0.2</v>
@@ -2217,7 +2295,7 @@
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B4" s="1">
         <v>1000</v>
@@ -2237,7 +2315,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B5" s="7">
         <v>10</v>
@@ -2265,10 +2343,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D9D62FD-4CBF-488C-B0DF-12E645A3B6BE}">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
@@ -2283,18 +2361,18 @@
     <col min="13" max="13" width="25.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D1" s="10" t="str" cm="1">
-        <f t="array" ref="D1:L1">TRANSPOSE(_xlfn.VSTACK(sensors[sensor_id],Pos[config_id]))</f>
+        <f t="array" ref="D1:O1">TRANSPOSE(_xlfn.VSTACK(sensors[sensor_id],Pos[config_id]))</f>
         <v>cam_d435</v>
       </c>
       <c r="E1" s="10" t="str">
@@ -2313,173 +2391,205 @@
         <v>Basler_ace_2</v>
       </c>
       <c r="J1" s="10" t="str">
+        <v>Basler_ace_2_0,0001_noice</v>
+      </c>
+      <c r="K1" s="10" t="str">
+        <v>Basler_ace_2_0,0005_noice</v>
+      </c>
+      <c r="L1" s="10" t="str">
+        <v>Basler_ace_2_0,00005_noice</v>
+      </c>
+      <c r="M1" s="10" t="str">
         <v>setup_front</v>
       </c>
-      <c r="K1" s="10" t="str">
+      <c r="N1" s="10" t="str">
         <v>setup_top</v>
       </c>
-      <c r="L1" s="10" t="str">
+      <c r="O1" s="10" t="str">
         <v>setup_iso</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
-      </c>
-      <c r="J2" t="s">
-        <v>48</v>
-      </c>
-      <c r="K2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L2" t="s">
-        <v>48</v>
+        <v>44</v>
+      </c>
+      <c r="M2" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2" t="s">
+        <v>44</v>
+      </c>
+      <c r="O2" t="s">
+        <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J3" t="s">
-        <v>48</v>
-      </c>
-      <c r="K3" t="s">
-        <v>48</v>
+        <v>44</v>
+      </c>
+      <c r="M3" t="s">
+        <v>44</v>
+      </c>
+      <c r="N3" t="s">
+        <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G4" t="s">
+        <v>44</v>
+      </c>
+      <c r="H4" t="s">
+        <v>44</v>
+      </c>
+      <c r="I4" t="s">
+        <v>44</v>
+      </c>
+      <c r="M4" t="s">
+        <v>44</v>
+      </c>
+      <c r="N4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>49</v>
-      </c>
-      <c r="B4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D4" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" t="s">
-        <v>48</v>
-      </c>
-      <c r="F4" t="s">
-        <v>48</v>
-      </c>
-      <c r="G4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H4" t="s">
-        <v>48</v>
-      </c>
-      <c r="I4" t="s">
-        <v>48</v>
-      </c>
-      <c r="J4" t="s">
-        <v>48</v>
-      </c>
-      <c r="K4" t="s">
-        <v>48</v>
-      </c>
-      <c r="L4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>53</v>
       </c>
       <c r="B5" t="s">
         <v>47</v>
       </c>
       <c r="C5" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="I5" t="s">
-        <v>48</v>
-      </c>
-      <c r="J5" t="s">
-        <v>48</v>
-      </c>
-      <c r="K5" t="s">
-        <v>48</v>
-      </c>
-      <c r="L5" t="s">
-        <v>48</v>
+        <v>44</v>
+      </c>
+      <c r="M5" t="s">
+        <v>44</v>
+      </c>
+      <c r="N5" t="s">
+        <v>44</v>
+      </c>
+      <c r="O5" t="s">
+        <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
         <v>47</v>
       </c>
       <c r="C6" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="F6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="I6" t="s">
-        <v>48</v>
-      </c>
-      <c r="J6" t="s">
-        <v>48</v>
-      </c>
-      <c r="K6" t="s">
-        <v>48</v>
-      </c>
-      <c r="L6" t="s">
-        <v>48</v>
+        <v>44</v>
+      </c>
+      <c r="M6" t="s">
+        <v>44</v>
+      </c>
+      <c r="N6" t="s">
+        <v>44</v>
+      </c>
+      <c r="O6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" t="s">
+        <v>44</v>
+      </c>
+      <c r="K7" t="s">
+        <v>44</v>
+      </c>
+      <c r="L7" t="s">
+        <v>44</v>
+      </c>
+      <c r="O7" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>